<commit_message>
modif binding securtiy label et suppr consrt 4d0cb28e8530432b3557039d9310661ef7769ee2
</commit_message>
<xml_diff>
--- a/cp-clarification-securitylabel/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/cp-clarification-securitylabel/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4211" uniqueCount="766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4210" uniqueCount="766">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-07T15:16:01+00:00</t>
+    <t>2026-06-05T09:56:42+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1247,8 +1247,7 @@
     <t>Use of the Health Care Privacy/Security Classification (HCS) system of security-tag use is recommended.</t>
   </si>
   <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-constr-bind-securityLabel:Les codes pour cet élément doivent provenir du ValueSet spécifié par le standard. Lorsqu’aucun code ne correspond au concept recherché, un code provenant de la terminologie de référence TRE_A07-StatusVisibiliteDocument, OID : 1.2.250.1.213.1.1.4.13 peut être utilisé. {null}</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J08-XdsConfidentialityCode-CISIS/FHIR/JDV-J08-XdsConfidentialityCode-CISIS</t>
   </si>
   <si>
     <t>niveauConfidentialite : [0..*] code</t>
@@ -7728,11 +7727,9 @@
       <c r="X39" t="s" s="2">
         <v>157</v>
       </c>
-      <c r="Y39" t="s" s="2">
-        <v>158</v>
-      </c>
+      <c r="Y39" s="2"/>
       <c r="Z39" t="s" s="2">
-        <v>159</v>
+        <v>392</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>82</v>
@@ -7762,7 +7759,7 @@
         <v>82</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>392</v>
+        <v>109</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>393</v>

</xml_diff>